<commit_message>
Clarify which CMS file supports 65+ figures and beneficiary-count limits
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/cms_medicare_adhd_older_americans/stimulant_growth_65plus.xlsx
+++ b/cms_medicare_adhd_older_americans/stimulant_growth_65plus.xlsx
@@ -1,17 +1,23 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <fileVersion appName="xl" lastEdited="4" lowestEdited="4" rupBuild="4505"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="30430"/>
   <workbookPr defaultThemeVersion="124226"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://manhattaninstituteny-my.sharepoint.com/personal/cgorman_manhattan_institute/Documents/Documents/research/repos/cms-medicare-adhd-older-americans/cms_medicare_adhd_older_americans/"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="1" documentId="11_7D22A20A6FF01BD845E2684A94C48437D2B2E360" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{E125748A-5E50-4428-9B4C-5C0A41EE1E8F}"/>
   <bookViews>
-    <workbookView xWindow="240" yWindow="15" windowWidth="16095" windowHeight="9660"/>
+    <workbookView xWindow="2304" yWindow="2304" windowWidth="17280" windowHeight="9960" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Growth" sheetId="1" r:id="rId1"/>
     <sheet name="Annual_65plus" sheetId="2" r:id="rId2"/>
     <sheet name="Ingredient_Year_65plus" sheetId="3" r:id="rId3"/>
   </sheets>
-  <calcPr calcId="124519" fullCalcOnLoad="1"/>
+  <calcPr calcId="124519"/>
 </workbook>
 </file>
 
@@ -141,8 +147,8 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <fonts count="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <fonts count="1" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -179,13 +185,21 @@
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    </ext>
+  </extLst>
 </styleSheet>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme 2007 - 2010">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2007 - 2010">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -223,7 +237,7 @@
         <a:srgbClr val="800080"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2007 - 2010">
       <a:majorFont>
         <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
@@ -257,6 +271,7 @@
         <a:font script="Mong" typeface="Mongolian Baiti"/>
         <a:font script="Viet" typeface="Times New Roman"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
+        <a:font script="Geor" typeface="Sylfaen"/>
       </a:majorFont>
       <a:minorFont>
         <a:latin typeface="Calibri"/>
@@ -291,9 +306,10 @@
         <a:font script="Mong" typeface="Mongolian Baiti"/>
         <a:font script="Viet" typeface="Arial"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
+        <a:font script="Geor" typeface="Sylfaen"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2007 - 2010">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -466,11 +482,20 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:G12"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="31.77734375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="20.44140625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="15.33203125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="20.44140625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="15.33203125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="20.44140625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="15.33203125" bestFit="1" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="1" spans="1:7">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -493,53 +518,53 @@
         <v>6</v>
       </c>
     </row>
-    <row r="2" spans="1:7">
+    <row r="2" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>7</v>
       </c>
       <c r="B2">
-        <v>2.211910101404056</v>
+        <v>2.2119101014040559</v>
       </c>
       <c r="C2">
         <v>0.1119093911814473</v>
       </c>
       <c r="D2">
-        <v>1.078909906396256</v>
+        <v>1.0789099063962559</v>
       </c>
       <c r="E2">
-        <v>0.1297246669610805</v>
+        <v>0.12972466696108051</v>
       </c>
       <c r="F2">
-        <v>0.544997256264862</v>
+        <v>0.54499725626486195</v>
       </c>
       <c r="G2">
-        <v>0.09090150901244964</v>
-      </c>
-    </row>
-    <row r="3" spans="1:7">
+        <v>9.0901509012449644E-2</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>8</v>
       </c>
       <c r="B3">
-        <v>2.118580097546632</v>
+        <v>2.1185800975466318</v>
       </c>
       <c r="C3">
         <v>0.1089326564311595</v>
       </c>
       <c r="D3">
-        <v>1.027249348231965</v>
+        <v>1.0272493482319649</v>
       </c>
       <c r="E3">
         <v>0.1249965611428769</v>
       </c>
       <c r="F3">
-        <v>0.5383307930356245</v>
+        <v>0.53833079303562448</v>
       </c>
       <c r="G3">
-        <v>0.08995846018283271</v>
-      </c>
-    </row>
-    <row r="4" spans="1:7">
+        <v>8.9958460182832711E-2</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>9</v>
       </c>
@@ -547,33 +572,33 @@
         <v>1.810876127946683</v>
       </c>
       <c r="C4">
-        <v>0.098509435435159</v>
+        <v>9.8509435435158998E-2</v>
       </c>
       <c r="D4">
-        <v>0.7632178029990597</v>
+        <v>0.76321780299905972</v>
       </c>
       <c r="E4">
-        <v>0.09913488934941572</v>
+        <v>9.9134889349415722E-2</v>
       </c>
       <c r="F4">
-        <v>0.5941740851105632</v>
+        <v>0.59417408511056324</v>
       </c>
       <c r="G4">
-        <v>0.09775936052082668</v>
-      </c>
-    </row>
-    <row r="5" spans="1:7">
+        <v>9.7759360520826677E-2</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>10</v>
       </c>
       <c r="B5">
-        <v>1.109861335720085</v>
+        <v>1.1098613357200851</v>
       </c>
       <c r="C5">
-        <v>0.07023125144573195</v>
+        <v>7.0231251445731946E-2</v>
       </c>
       <c r="D5">
-        <v>0.8603619700710936</v>
+        <v>0.86036197007109361</v>
       </c>
       <c r="E5">
         <v>0.109003479705007</v>
@@ -582,168 +607,168 @@
         <v>0.1341133444259002</v>
       </c>
       <c r="G5">
-        <v>0.02548967504153499</v>
-      </c>
-    </row>
-    <row r="6" spans="1:7">
+        <v>2.5489675041534991E-2</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>11</v>
       </c>
       <c r="B6">
-        <v>0.566860703388846</v>
+        <v>0.56686070338884598</v>
       </c>
       <c r="C6">
-        <v>0.04166970889486321</v>
+        <v>4.1669708894863211E-2</v>
       </c>
       <c r="D6">
-        <v>0.6951788664572129</v>
+        <v>0.69517886645721294</v>
       </c>
       <c r="E6">
-        <v>0.09194958666543473</v>
+        <v>9.1949586665434735E-2</v>
       </c>
       <c r="F6">
-        <v>-0.07569594312872818</v>
+        <v>-7.5695943128728183E-2</v>
       </c>
       <c r="G6">
-        <v>-0.0156195683518261</v>
-      </c>
-    </row>
-    <row r="7" spans="1:7">
+        <v>-1.56195683518261E-2</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>12</v>
       </c>
       <c r="B7">
-        <v>-0.3234544986098322</v>
+        <v>-0.32345449860983222</v>
       </c>
       <c r="C7">
-        <v>-0.03489968913890484</v>
+        <v>-3.4899689138904837E-2</v>
       </c>
       <c r="D7">
-        <v>-0.08232207760057753</v>
+        <v>-8.2322077600577526E-2</v>
       </c>
       <c r="E7">
-        <v>-0.01421611584449889</v>
+        <v>-1.4216115844498891E-2</v>
       </c>
       <c r="F7">
-        <v>-0.2627636724426951</v>
+        <v>-0.26276367244269511</v>
       </c>
       <c r="G7">
-        <v>-0.05914792856462026</v>
-      </c>
-    </row>
-    <row r="8" spans="1:7">
+        <v>-5.9147928564620263E-2</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>13</v>
       </c>
       <c r="B8">
-        <v>-0.4975724033442381</v>
+        <v>-0.49757240334423808</v>
       </c>
       <c r="C8">
-        <v>-0.06065557466110372</v>
+        <v>-6.0655574661103717E-2</v>
       </c>
       <c r="D8">
         <v>-0.1638034719628165</v>
       </c>
       <c r="E8">
-        <v>-0.02937517821731839</v>
+        <v>-2.9375178217318391E-2</v>
       </c>
       <c r="F8">
-        <v>-0.399151300191215</v>
+        <v>-0.39915130019121497</v>
       </c>
       <c r="G8">
-        <v>-0.09686426812719895</v>
-      </c>
-    </row>
-    <row r="9" spans="1:7">
+        <v>-9.6864268127198949E-2</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
         <v>14</v>
       </c>
       <c r="B9">
-        <v>0.3976135937067593</v>
+        <v>0.39761359370675931</v>
       </c>
       <c r="C9">
-        <v>0.03090111786476846</v>
+        <v>3.090111786476846E-2</v>
       </c>
       <c r="D9">
-        <v>0.3158354408529083</v>
+        <v>0.31583544085290832</v>
       </c>
       <c r="E9">
-        <v>0.04680775159955974</v>
+        <v>4.6807751599559737E-2</v>
       </c>
       <c r="F9">
-        <v>0.06214922498275577</v>
+        <v>6.2149224982755769E-2</v>
       </c>
       <c r="G9">
-        <v>0.01213188672322607</v>
-      </c>
-    </row>
-    <row r="10" spans="1:7">
+        <v>1.2131886723226071E-2</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
         <v>15</v>
       </c>
       <c r="B10">
-        <v>0.05004651615792977</v>
+        <v>5.0046516157929773E-2</v>
       </c>
       <c r="C10">
-        <v>0.004449365918740567</v>
+        <v>4.4493659187405674E-3</v>
       </c>
       <c r="D10">
         <v>0.1511644249052497</v>
       </c>
       <c r="E10">
-        <v>0.02373973463446699</v>
+        <v>2.3739734634466991E-2</v>
       </c>
       <c r="F10">
-        <v>-0.08783967481938371</v>
+        <v>-8.7839674819383706E-2</v>
       </c>
       <c r="G10">
-        <v>-0.01821987583179929</v>
-      </c>
-    </row>
-    <row r="11" spans="1:7">
+        <v>-1.8219875831799289E-2</v>
+      </c>
+    </row>
+    <row r="11" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
         <v>16</v>
       </c>
       <c r="B11">
-        <v>0.9356324431221865</v>
+        <v>0.93563244312218652</v>
       </c>
       <c r="C11">
-        <v>0.06187845295146954</v>
+        <v>6.1878452951469542E-2</v>
       </c>
       <c r="D11">
         <v>0.5421036045022305</v>
       </c>
       <c r="E11">
-        <v>0.07486088461628881</v>
+        <v>7.4860884616288814E-2</v>
       </c>
       <c r="F11">
-        <v>0.2551896237522779</v>
+        <v>0.25518962375227788</v>
       </c>
       <c r="G11">
-        <v>0.0465063504478842</v>
-      </c>
-    </row>
-    <row r="12" spans="1:7">
+        <v>4.6506350447884197E-2</v>
+      </c>
+    </row>
+    <row r="12" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
         <v>17</v>
       </c>
       <c r="B12">
-        <v>0.3403079459743554</v>
+        <v>0.34030794597435537</v>
       </c>
       <c r="C12">
-        <v>0.02698488991416248</v>
+        <v>2.698488991416248E-2</v>
       </c>
       <c r="D12">
-        <v>0.3452800477615219</v>
+        <v>0.34528004776152188</v>
       </c>
       <c r="E12">
-        <v>0.05067593102462609</v>
+        <v>5.0675931024626093E-2</v>
       </c>
       <c r="F12">
-        <v>-0.003695960402772425</v>
+        <v>-3.6959604027724251E-3</v>
       </c>
       <c r="G12">
-        <v>-0.0007402873200950122</v>
+        <v>-7.4028732009501219E-4</v>
       </c>
     </row>
   </sheetData>
@@ -752,11 +777,11 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:U13"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
-    <row r="1" spans="1:21">
+    <row r="1" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>18</v>
       </c>
@@ -821,7 +846,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="2" spans="1:21">
+    <row r="2" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A2">
         <v>2013</v>
       </c>
@@ -835,19 +860,19 @@
         <v>121238</v>
       </c>
       <c r="E2">
-        <v>65164805.28</v>
+        <v>65164805.280000001</v>
       </c>
       <c r="F2">
         <v>1459852</v>
       </c>
       <c r="G2">
-        <v>172868791.36</v>
+        <v>172868791.36000001</v>
       </c>
       <c r="H2">
         <v>2075238</v>
       </c>
       <c r="I2">
-        <v>238042934.49</v>
+        <v>238042934.49000001</v>
       </c>
       <c r="J2">
         <v>30</v>
@@ -856,25 +881,25 @@
         <v>2</v>
       </c>
       <c r="L2">
-        <v>87747878.80801144</v>
+        <v>87747878.808011442</v>
       </c>
       <c r="M2">
-        <v>105.8970444617785</v>
+        <v>105.89704446177851</v>
       </c>
       <c r="N2">
-        <v>94.48270298037889</v>
+        <v>94.482702980378889</v>
       </c>
       <c r="O2">
         <v>127.2259885524456</v>
       </c>
       <c r="P2">
-        <v>0.2965250250814606</v>
+        <v>0.29652502508146061</v>
       </c>
       <c r="Q2">
-        <v>0.2737523187554954</v>
-      </c>
-    </row>
-    <row r="3" spans="1:21">
+        <v>0.27375231875549538</v>
+      </c>
+    </row>
+    <row r="3" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A3">
         <v>2014</v>
       </c>
@@ -888,7 +913,7 @@
         <v>135088</v>
       </c>
       <c r="E3">
-        <v>80558300.72</v>
+        <v>80558300.719999999</v>
       </c>
       <c r="F3">
         <v>1605452</v>
@@ -900,7 +925,7 @@
         <v>2329207</v>
       </c>
       <c r="I3">
-        <v>263522944.23</v>
+        <v>263522944.22999999</v>
       </c>
       <c r="J3">
         <v>29</v>
@@ -909,37 +934,37 @@
         <v>1</v>
       </c>
       <c r="L3">
-        <v>106744444.4214487</v>
+        <v>106744444.42144869</v>
       </c>
       <c r="M3">
-        <v>111.308651362786</v>
+        <v>111.30865136278599</v>
       </c>
       <c r="N3">
-        <v>98.92624291301196</v>
+        <v>98.926242913011961</v>
       </c>
       <c r="O3">
-        <v>131.0830385456366</v>
+        <v>131.08303854563661</v>
       </c>
       <c r="P3">
-        <v>0.3107229198607079</v>
+        <v>0.31072291986070788</v>
       </c>
       <c r="Q3">
-        <v>0.3056974828335615</v>
+        <v>0.30569748283356152</v>
       </c>
       <c r="R3">
-        <v>0.1761212948517941</v>
+        <v>0.17612129485179409</v>
       </c>
       <c r="S3">
-        <v>0.1806957189703537</v>
+        <v>0.18069571897035369</v>
       </c>
       <c r="T3">
-        <v>0.2362240687109745</v>
+        <v>0.23622406871097451</v>
       </c>
       <c r="U3">
-        <v>0.2164903114638352</v>
-      </c>
-    </row>
-    <row r="4" spans="1:21">
+        <v>0.21649031146383521</v>
+      </c>
+    </row>
+    <row r="4" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A4">
         <v>2015</v>
       </c>
@@ -947,25 +972,25 @@
         <v>811782</v>
       </c>
       <c r="C4">
-        <v>910054.4</v>
+        <v>910054.40000000002</v>
       </c>
       <c r="D4">
         <v>149020</v>
       </c>
       <c r="E4">
-        <v>91919444.36</v>
+        <v>91919444.359999999</v>
       </c>
       <c r="F4">
         <v>1712881</v>
       </c>
       <c r="G4">
-        <v>195233693.46</v>
+        <v>195233693.46000001</v>
       </c>
       <c r="H4">
         <v>2524674</v>
       </c>
       <c r="I4">
-        <v>287155922.67</v>
+        <v>287155922.67000002</v>
       </c>
       <c r="J4">
         <v>30</v>
@@ -977,34 +1002,34 @@
         <v>121654221.3505531</v>
       </c>
       <c r="M4">
-        <v>113.2316857974185</v>
+        <v>113.23168579741851</v>
       </c>
       <c r="N4">
-        <v>101.0043403559172</v>
+        <v>101.00434035591719</v>
       </c>
       <c r="O4">
         <v>133.6779662298793</v>
       </c>
       <c r="P4">
-        <v>0.3215393353755772</v>
+        <v>0.32153933537557722</v>
       </c>
       <c r="Q4">
-        <v>0.3201029026506758</v>
+        <v>0.32010290265067581</v>
       </c>
       <c r="R4">
         <v>0.1216517579566085</v>
       </c>
       <c r="S4">
-        <v>0.1175541419545394</v>
+        <v>0.11755414195453941</v>
       </c>
       <c r="T4">
-        <v>0.1410300805560487</v>
+        <v>0.14103008055604871</v>
       </c>
       <c r="U4">
-        <v>0.1396773107014126</v>
-      </c>
-    </row>
-    <row r="5" spans="1:21">
+        <v>0.13967731070141259</v>
+      </c>
+    </row>
+    <row r="5" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A5">
         <v>2016</v>
       </c>
@@ -1024,13 +1049,13 @@
         <v>1815510</v>
       </c>
       <c r="G5">
-        <v>191684524.29</v>
+        <v>191684524.28999999</v>
       </c>
       <c r="H5">
         <v>2763486</v>
       </c>
       <c r="I5">
-        <v>291891923.39</v>
+        <v>291891923.38999999</v>
       </c>
       <c r="J5">
         <v>32</v>
@@ -1039,37 +1064,37 @@
         <v>1</v>
       </c>
       <c r="L5">
-        <v>130961858.2676071</v>
+        <v>130961858.26760709</v>
       </c>
       <c r="M5">
-        <v>105.7016400778518</v>
+        <v>105.70164007785181</v>
       </c>
       <c r="N5">
-        <v>94.7810365466468</v>
+        <v>94.781036546646803</v>
       </c>
       <c r="O5">
-        <v>123.8787559249567</v>
+        <v>123.87875592495671</v>
       </c>
       <c r="P5">
-        <v>0.3430286963639403</v>
+        <v>0.34302869636394029</v>
       </c>
       <c r="Q5">
-        <v>0.3432791050066882</v>
+        <v>0.34327910500668818</v>
       </c>
       <c r="R5">
-        <v>0.1677457741117689</v>
+        <v>0.16774577411176891</v>
       </c>
       <c r="S5">
-        <v>0.1616642917170665</v>
+        <v>0.16166429171706651</v>
       </c>
       <c r="T5">
-        <v>0.09008925062218465</v>
+        <v>9.0089250622184647E-2</v>
       </c>
       <c r="U5">
-        <v>0.07650895146690861</v>
-      </c>
-    </row>
-    <row r="6" spans="1:21">
+        <v>7.6508951466908615E-2</v>
+      </c>
+    </row>
+    <row r="6" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A6">
         <v>2017</v>
       </c>
@@ -1089,13 +1114,13 @@
         <v>1865281</v>
       </c>
       <c r="G6">
-        <v>196266095.73</v>
+        <v>196266095.72999999</v>
       </c>
       <c r="H6">
         <v>2935808</v>
       </c>
       <c r="I6">
-        <v>303302100.17</v>
+        <v>303302100.17000002</v>
       </c>
       <c r="J6">
         <v>34</v>
@@ -1104,37 +1129,37 @@
         <v>3</v>
       </c>
       <c r="L6">
-        <v>136925502.3101313</v>
+        <v>136925502.31013131</v>
       </c>
       <c r="M6">
-        <v>99.95672546323198</v>
+        <v>99.956725463231976</v>
       </c>
       <c r="N6">
-        <v>91.28792309312726</v>
+        <v>91.287923093127262</v>
       </c>
       <c r="O6">
-        <v>116.8244831395235</v>
+        <v>116.82448313952349</v>
       </c>
       <c r="P6">
-        <v>0.3646062685298221</v>
+        <v>0.36460626852982209</v>
       </c>
       <c r="Q6">
-        <v>0.3527673506712599</v>
+        <v>0.35276735067125992</v>
       </c>
       <c r="R6">
-        <v>0.129182292408395</v>
+        <v>0.12918229240839499</v>
       </c>
       <c r="S6">
         <v>0.1086704723340268</v>
       </c>
       <c r="T6">
-        <v>0.06781090924490729</v>
+        <v>6.7810909244907291E-2</v>
       </c>
       <c r="U6">
-        <v>0.04553725887378635</v>
-      </c>
-    </row>
-    <row r="7" spans="1:21">
+        <v>4.5537258873786353E-2</v>
+      </c>
+    </row>
+    <row r="7" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A7">
         <v>2018</v>
       </c>
@@ -1160,7 +1185,7 @@
         <v>3090049</v>
       </c>
       <c r="I7">
-        <v>314645008.43</v>
+        <v>314645008.43000001</v>
       </c>
       <c r="J7">
         <v>37</v>
@@ -1169,19 +1194,19 @@
         <v>5</v>
       </c>
       <c r="L7">
-        <v>143038246.5445214</v>
+        <v>143038246.54452139</v>
       </c>
       <c r="M7">
         <v>96.98096242697946</v>
       </c>
       <c r="N7">
-        <v>88.55676587589315</v>
+        <v>88.556765875893149</v>
       </c>
       <c r="O7">
         <v>110.6272757463673</v>
       </c>
       <c r="P7">
-        <v>0.3820848795601623</v>
+        <v>0.38208487956016229</v>
       </c>
       <c r="Q7">
         <v>0.363907378195302</v>
@@ -1190,16 +1215,16 @@
         <v>0.1029947291421824</v>
       </c>
       <c r="S7">
-        <v>0.1031624870943229</v>
+        <v>0.10316248709432289</v>
       </c>
       <c r="T7">
-        <v>0.0701580097623542</v>
+        <v>7.0158009762354201E-2</v>
       </c>
       <c r="U7">
-        <v>0.04464284688578291</v>
-      </c>
-    </row>
-    <row r="8" spans="1:21">
+        <v>4.4642846885782912E-2</v>
+      </c>
+    </row>
+    <row r="8" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A8">
         <v>2019</v>
       </c>
@@ -1219,13 +1244,13 @@
         <v>1920925</v>
       </c>
       <c r="G8">
-        <v>199000402.79</v>
+        <v>199000402.78999999</v>
       </c>
       <c r="H8">
         <v>3200232</v>
       </c>
       <c r="I8">
-        <v>320234410.28</v>
+        <v>320234410.27999997</v>
       </c>
       <c r="J8">
         <v>37</v>
@@ -1234,37 +1259,37 @@
         <v>5</v>
       </c>
       <c r="L8">
-        <v>148748349.7317897</v>
+        <v>148748349.73178971</v>
       </c>
       <c r="M8">
         <v>94.76448866469994</v>
       </c>
       <c r="N8">
-        <v>86.70469057371582</v>
+        <v>86.704690573715823</v>
       </c>
       <c r="O8">
         <v>106.3859299036535</v>
       </c>
       <c r="P8">
-        <v>0.3997453934589743</v>
+        <v>0.39974539345897431</v>
       </c>
       <c r="Q8">
-        <v>0.3785668299168765</v>
+        <v>0.37856682991687651</v>
       </c>
       <c r="R8">
-        <v>0.08352693957029156</v>
+        <v>8.3526939570291558E-2</v>
       </c>
       <c r="S8">
-        <v>0.08137917646481041</v>
+        <v>8.137917646481041E-2</v>
       </c>
       <c r="T8">
-        <v>0.0587632233503288</v>
+        <v>5.8763223350328797E-2</v>
       </c>
       <c r="U8">
-        <v>0.03992011455125799</v>
-      </c>
-    </row>
-    <row r="9" spans="1:21">
+        <v>3.992011455125799E-2</v>
+      </c>
+    </row>
+    <row r="9" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A9">
         <v>2020</v>
       </c>
@@ -1278,19 +1303,19 @@
         <v>224082</v>
       </c>
       <c r="E9">
-        <v>121929034.68</v>
+        <v>121929034.68000001</v>
       </c>
       <c r="F9">
         <v>1976485</v>
       </c>
       <c r="G9">
-        <v>193725070.9</v>
+        <v>193725070.90000001</v>
       </c>
       <c r="H9">
         <v>3372358</v>
       </c>
       <c r="I9">
-        <v>315655051.57</v>
+        <v>315655051.56999999</v>
       </c>
       <c r="J9">
         <v>37</v>
@@ -1299,37 +1324,37 @@
         <v>6</v>
       </c>
       <c r="L9">
-        <v>147782733.1903765</v>
+        <v>147782733.19037649</v>
       </c>
       <c r="M9">
-        <v>87.35053804144975</v>
+        <v>87.350538041449752</v>
       </c>
       <c r="N9">
-        <v>79.42968777299488</v>
+        <v>79.429687772994882</v>
       </c>
       <c r="O9">
-        <v>96.27187147309424</v>
+        <v>96.271871473094237</v>
       </c>
       <c r="P9">
-        <v>0.413911868194302</v>
+        <v>0.41391186819430198</v>
       </c>
       <c r="Q9">
-        <v>0.386273034673614</v>
+        <v>0.38627303467361401</v>
       </c>
       <c r="R9">
-        <v>0.09113030944016853</v>
+        <v>9.1130309440168533E-2</v>
       </c>
       <c r="S9">
-        <v>0.09788365105113694</v>
+        <v>9.7883651051136944E-2</v>
       </c>
       <c r="T9">
-        <v>0.005765144158223601</v>
+        <v>5.7651441582236007E-3</v>
       </c>
       <c r="U9">
-        <v>-0.006491611793706609</v>
-      </c>
-    </row>
-    <row r="10" spans="1:21">
+        <v>-6.4916117937066087E-3</v>
+      </c>
+    </row>
+    <row r="10" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A10">
         <v>2021</v>
       </c>
@@ -1349,13 +1374,13 @@
         <v>1952129</v>
       </c>
       <c r="G10">
-        <v>197195074.14</v>
+        <v>197195074.13999999</v>
       </c>
       <c r="H10">
         <v>3418655</v>
       </c>
       <c r="I10">
-        <v>322676110.07</v>
+        <v>322676110.06999999</v>
       </c>
       <c r="J10">
         <v>37</v>
@@ -1367,34 +1392,34 @@
         <v>145242696.7993083</v>
       </c>
       <c r="M10">
-        <v>85.55447815197164</v>
+        <v>85.554478151971637</v>
       </c>
       <c r="N10">
-        <v>77.36421299743994</v>
+        <v>77.364212997439935</v>
       </c>
       <c r="O10">
-        <v>89.5608466286081</v>
+        <v>89.560846628608104</v>
       </c>
       <c r="P10">
-        <v>0.4289613897863341</v>
+        <v>0.42896138978633408</v>
       </c>
       <c r="Q10">
-        <v>0.388820731422548</v>
+        <v>0.38882073142254803</v>
       </c>
       <c r="R10">
-        <v>0.05058677129996658</v>
+        <v>5.0586771299966582E-2</v>
       </c>
       <c r="S10">
-        <v>0.05645702092210048</v>
+        <v>5.6457020922100483E-2</v>
       </c>
       <c r="T10">
-        <v>0.02898510973432389</v>
+        <v>2.8985109734323888E-2</v>
       </c>
       <c r="U10">
-        <v>-0.01718763982931648</v>
-      </c>
-    </row>
-    <row r="11" spans="1:21">
+        <v>-1.7187639829316481E-2</v>
+      </c>
+    </row>
+    <row r="11" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A11">
         <v>2022</v>
       </c>
@@ -1414,7 +1439,7 @@
         <v>1970492</v>
       </c>
       <c r="G11">
-        <v>206835610.54</v>
+        <v>206835610.53999999</v>
       </c>
       <c r="H11">
         <v>3543134</v>
@@ -1429,37 +1454,37 @@
         <v>7</v>
       </c>
       <c r="L11">
-        <v>143593763.2556962</v>
+        <v>143593763.25569621</v>
       </c>
       <c r="M11">
-        <v>85.1857714585486</v>
+        <v>85.185771458548601</v>
       </c>
       <c r="N11">
         <v>77.03416225943873</v>
       </c>
       <c r="O11">
-        <v>82.57084049478424</v>
+        <v>82.570840494784235</v>
       </c>
       <c r="P11">
-        <v>0.4438514038701331</v>
+        <v>0.44385140387013311</v>
       </c>
       <c r="Q11">
-        <v>0.3930866443740844</v>
+        <v>0.39308664437408442</v>
       </c>
       <c r="R11">
-        <v>0.0723873844078744</v>
+        <v>7.23873844078744E-2</v>
       </c>
       <c r="S11">
-        <v>0.07234062285316778</v>
+        <v>7.234062285316778E-2</v>
       </c>
       <c r="T11">
-        <v>0.06776580976778068</v>
+        <v>6.7765809767780683E-2</v>
       </c>
       <c r="U11">
-        <v>-0.01135295322897056</v>
-      </c>
-    </row>
-    <row r="12" spans="1:21">
+        <v>-1.135295322897056E-2</v>
+      </c>
+    </row>
+    <row r="12" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A12">
         <v>2023</v>
       </c>
@@ -1485,7 +1510,7 @@
         <v>3620954</v>
       </c>
       <c r="I12">
-        <v>382804260.59</v>
+        <v>382804260.58999997</v>
       </c>
       <c r="J12">
         <v>38</v>
@@ -1494,28 +1519,28 @@
         <v>2</v>
       </c>
       <c r="L12">
-        <v>158727303.2640088</v>
+        <v>158727303.26400879</v>
       </c>
       <c r="M12">
         <v>91.82187926525755</v>
       </c>
       <c r="N12">
-        <v>84.36441283399566</v>
+        <v>84.364412833995658</v>
       </c>
       <c r="O12">
-        <v>86.85268983296226</v>
+        <v>86.852689832962255</v>
       </c>
       <c r="P12">
         <v>0.4637228200082078</v>
       </c>
       <c r="Q12">
-        <v>0.4027642269507897</v>
+        <v>0.40276422695078973</v>
       </c>
       <c r="R12">
-        <v>0.06771735156187897</v>
+        <v>6.7717351561878969E-2</v>
       </c>
       <c r="S12">
-        <v>0.05089540350258193</v>
+        <v>5.0895403502581933E-2</v>
       </c>
       <c r="T12">
         <v>0.150894240504021</v>
@@ -1524,7 +1549,7 @@
         <v>0.1053913461503508</v>
       </c>
     </row>
-    <row r="13" spans="1:21">
+    <row r="13" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A13">
         <v>2024</v>
       </c>
@@ -1538,7 +1563,7 @@
         <v>340785</v>
       </c>
       <c r="E13">
-        <v>137488703.11</v>
+        <v>137488703.11000001</v>
       </c>
       <c r="F13">
         <v>2040309</v>
@@ -1550,7 +1575,7 @@
         <v>4016898</v>
       </c>
       <c r="I13">
-        <v>319050836.58</v>
+        <v>319050836.57999998</v>
       </c>
       <c r="J13">
         <v>38</v>
@@ -1559,34 +1584,34 @@
         <v>7</v>
       </c>
       <c r="L13">
-        <v>137488703.11</v>
+        <v>137488703.11000001</v>
       </c>
       <c r="M13">
-        <v>69.56237024793055</v>
+        <v>69.562370247930545</v>
       </c>
       <c r="N13">
-        <v>63.92184766055873</v>
+        <v>63.921847660558733</v>
       </c>
       <c r="O13">
-        <v>63.92184766055873</v>
+        <v>63.921847660558733</v>
       </c>
       <c r="P13">
         <v>0.4920416201755683</v>
       </c>
       <c r="Q13">
-        <v>0.4309303952429085</v>
+        <v>0.43093039524290849</v>
       </c>
       <c r="R13">
-        <v>0.177094059444268</v>
+        <v>0.17709405944426801</v>
       </c>
       <c r="S13">
-        <v>0.1769264711338077</v>
+        <v>0.17692647113380769</v>
       </c>
       <c r="T13">
         <v>-0.1082577111805743</v>
       </c>
       <c r="U13">
-        <v>-0.1338055880574179</v>
+        <v>-0.13380558805741791</v>
       </c>
     </row>
   </sheetData>
@@ -1595,11 +1620,11 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1:H71"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
-    <row r="1" spans="1:8">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>18</v>
       </c>
@@ -1625,7 +1650,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="2" spans="1:8">
+    <row r="2" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A2">
         <v>2013</v>
       </c>
@@ -1642,16 +1667,16 @@
         <v>1032891.11</v>
       </c>
       <c r="F2">
-        <v>150.4509795638938</v>
+        <v>150.45097956389381</v>
       </c>
       <c r="G2">
-        <v>0.009646385855434217</v>
+        <v>9.6463858554342169E-3</v>
       </c>
       <c r="H2">
-        <v>0.01585044420161889</v>
-      </c>
-    </row>
-    <row r="3" spans="1:8">
+        <v>1.585044420161889E-2</v>
+      </c>
+    </row>
+    <row r="3" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A3">
         <v>2013</v>
       </c>
@@ -1665,19 +1690,19 @@
         <v>24609.8</v>
       </c>
       <c r="E3">
-        <v>4750617.48</v>
+        <v>4750617.4800000004</v>
       </c>
       <c r="F3">
-        <v>193.0376305374282</v>
+        <v>193.03763053742821</v>
       </c>
       <c r="G3">
-        <v>0.03516478159126365</v>
+        <v>3.5164781591263648E-2</v>
       </c>
       <c r="H3">
-        <v>0.07290158329465664</v>
-      </c>
-    </row>
-    <row r="4" spans="1:8">
+        <v>7.2901583294656638E-2</v>
+      </c>
+    </row>
+    <row r="4" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A4">
         <v>2013</v>
       </c>
@@ -1691,19 +1716,19 @@
         <v>1306.3</v>
       </c>
       <c r="E4">
-        <v>801063.7000000001</v>
+        <v>801063.70000000007</v>
       </c>
       <c r="F4">
-        <v>613.2310342187859</v>
+        <v>613.23103421878591</v>
       </c>
       <c r="G4">
-        <v>0.001847698907956318</v>
+        <v>1.847698907956318E-3</v>
       </c>
       <c r="H4">
-        <v>0.01229288872356775</v>
-      </c>
-    </row>
-    <row r="5" spans="1:8">
+        <v>1.2292888723567749E-2</v>
+      </c>
+    </row>
+    <row r="5" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A5">
         <v>2013</v>
       </c>
@@ -1717,19 +1742,19 @@
         <v>366563.5</v>
       </c>
       <c r="E5">
-        <v>21360711.45</v>
+        <v>21360711.449999999</v>
       </c>
       <c r="F5">
-        <v>58.27288164260762</v>
+        <v>58.272881642607622</v>
       </c>
       <c r="G5">
-        <v>0.5326101794071763</v>
+        <v>0.53261017940717625</v>
       </c>
       <c r="H5">
-        <v>0.3277952164242238</v>
-      </c>
-    </row>
-    <row r="6" spans="1:8">
+        <v>0.32779521642422382</v>
+      </c>
+    </row>
+    <row r="6" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A6">
         <v>2013</v>
       </c>
@@ -1743,19 +1768,19 @@
         <v>290356</v>
       </c>
       <c r="E6">
-        <v>37219521.54</v>
+        <v>37219521.539999999</v>
       </c>
       <c r="F6">
-        <v>128.1858185813277</v>
+        <v>128.18581858132771</v>
       </c>
       <c r="G6">
-        <v>0.4207309542381695</v>
+        <v>0.42073095423816947</v>
       </c>
       <c r="H6">
-        <v>0.571159867355933</v>
-      </c>
-    </row>
-    <row r="7" spans="1:8">
+        <v>0.57115986735593305</v>
+      </c>
+    </row>
+    <row r="7" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A7">
         <v>2014</v>
       </c>
@@ -1772,16 +1797,16 @@
         <v>1228186.21</v>
       </c>
       <c r="F7">
-        <v>168.6953107616235</v>
+        <v>168.69531076162349</v>
       </c>
       <c r="G7">
-        <v>0.008428464444315484</v>
+        <v>8.4284644443154838E-3</v>
       </c>
       <c r="H7">
-        <v>0.01524592995411932</v>
-      </c>
-    </row>
-    <row r="8" spans="1:8">
+        <v>1.524592995411932E-2</v>
+      </c>
+    </row>
+    <row r="8" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A8">
         <v>2014</v>
       </c>
@@ -1798,16 +1823,16 @@
         <v>6931844.54</v>
       </c>
       <c r="F8">
-        <v>215.8048043485705</v>
+        <v>215.80480434857051</v>
       </c>
       <c r="G8">
-        <v>0.0388925274063266</v>
+        <v>3.88925274063266E-2</v>
       </c>
       <c r="H8">
-        <v>0.08604755162467136</v>
-      </c>
-    </row>
-    <row r="9" spans="1:8">
+        <v>8.6047551624671356E-2</v>
+      </c>
+    </row>
+    <row r="9" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A9">
         <v>2014</v>
       </c>
@@ -1824,16 +1849,16 @@
         <v>868420.13</v>
       </c>
       <c r="F9">
-        <v>607.2868041958042</v>
+        <v>607.28680419580417</v>
       </c>
       <c r="G9">
-        <v>0.001698128328207169</v>
+        <v>1.698128328207169E-3</v>
       </c>
       <c r="H9">
-        <v>0.01078002046019324</v>
-      </c>
-    </row>
-    <row r="10" spans="1:8">
+        <v>1.0780020460193241E-2</v>
+      </c>
+    </row>
+    <row r="10" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A10">
         <v>2014</v>
       </c>
@@ -1847,19 +1872,19 @@
         <v>411055.3</v>
       </c>
       <c r="E10">
-        <v>30249679.06</v>
+        <v>30249679.059999999</v>
       </c>
       <c r="F10">
-        <v>73.59029079542339</v>
+        <v>73.590290795423385</v>
       </c>
       <c r="G10">
-        <v>0.5036947072006721</v>
+        <v>0.50369470720067211</v>
       </c>
       <c r="H10">
-        <v>0.375500461028096</v>
-      </c>
-    </row>
-    <row r="11" spans="1:8">
+        <v>0.37550046102809598</v>
+      </c>
+    </row>
+    <row r="11" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A11">
         <v>2014</v>
       </c>
@@ -1873,19 +1898,19 @@
         <v>362440.2</v>
       </c>
       <c r="E11">
-        <v>41280170.78</v>
+        <v>41280170.780000001</v>
       </c>
       <c r="F11">
         <v>113.8951219539113</v>
       </c>
       <c r="G11">
-        <v>0.4472861726204787</v>
+        <v>0.44728617262047871</v>
       </c>
       <c r="H11">
         <v>0.5124260369329201</v>
       </c>
     </row>
-    <row r="12" spans="1:8">
+    <row r="12" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A12">
         <v>2015</v>
       </c>
@@ -1902,16 +1927,16 @@
         <v>28890.07</v>
       </c>
       <c r="F12">
-        <v>321.0007777777778</v>
+        <v>321.00077777777778</v>
       </c>
       <c r="G12">
-        <v>0.0001059397720077558</v>
+        <v>1.0593977200775579E-4</v>
       </c>
       <c r="H12">
-        <v>0.0003142977005697818</v>
-      </c>
-    </row>
-    <row r="13" spans="1:8">
+        <v>3.1429770056978182E-4</v>
+      </c>
+    </row>
+    <row r="13" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A13">
         <v>2015</v>
       </c>
@@ -1922,22 +1947,22 @@
         <v>7025</v>
       </c>
       <c r="D13">
-        <v>8286.700000000001</v>
+        <v>8286.7000000000007</v>
       </c>
       <c r="E13">
-        <v>1295528.66</v>
+        <v>1295528.6599999999</v>
       </c>
       <c r="F13">
         <v>156.338308373659</v>
       </c>
       <c r="G13">
-        <v>0.008653801143656794</v>
+        <v>8.653801143656794E-3</v>
       </c>
       <c r="H13">
-        <v>0.01409417418719479</v>
-      </c>
-    </row>
-    <row r="14" spans="1:8">
+        <v>1.409417418719479E-2</v>
+      </c>
+    </row>
+    <row r="14" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A14">
         <v>2015</v>
       </c>
@@ -1951,19 +1976,19 @@
         <v>42680.3</v>
       </c>
       <c r="E14">
-        <v>10058876.61</v>
+        <v>10058876.609999999</v>
       </c>
       <c r="F14">
         <v>235.6796135453593</v>
       </c>
       <c r="G14">
-        <v>0.04639176527688468</v>
+        <v>4.6391765276884683E-2</v>
       </c>
       <c r="H14">
-        <v>0.1094314340130765</v>
-      </c>
-    </row>
-    <row r="15" spans="1:8">
+        <v>0.10943143401307651</v>
+      </c>
+    </row>
+    <row r="15" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A15">
         <v>2015</v>
       </c>
@@ -1980,16 +2005,16 @@
         <v>744020.51</v>
       </c>
       <c r="F15">
-        <v>665.3138782079943</v>
+        <v>665.31387820799432</v>
       </c>
       <c r="G15">
-        <v>0.001175192354597663</v>
+        <v>1.1751923545976629E-3</v>
       </c>
       <c r="H15">
-        <v>0.008094266835274415</v>
-      </c>
-    </row>
-    <row r="16" spans="1:8">
+        <v>8.0942668352744149E-3</v>
+      </c>
+    </row>
+    <row r="16" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A16">
         <v>2015</v>
       </c>
@@ -2003,19 +2028,19 @@
         <v>428136.1</v>
       </c>
       <c r="E16">
-        <v>36111812.67</v>
+        <v>36111812.670000002</v>
       </c>
       <c r="F16">
-        <v>84.34657266696267</v>
+        <v>84.346572666962672</v>
       </c>
       <c r="G16">
-        <v>0.4688253742999968</v>
+        <v>0.46882537429999682</v>
       </c>
       <c r="H16">
-        <v>0.3928636962661465</v>
-      </c>
-    </row>
-    <row r="17" spans="1:8">
+        <v>0.39286369626614648</v>
+      </c>
+    </row>
+    <row r="17" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A17">
         <v>2015</v>
       </c>
@@ -2029,19 +2054,19 @@
         <v>429743</v>
       </c>
       <c r="E17">
-        <v>43680315.84</v>
+        <v>43680315.840000004</v>
       </c>
       <c r="F17">
-        <v>101.6428792092018</v>
+        <v>101.64287920920179</v>
       </c>
       <c r="G17">
-        <v>0.4748479271528563</v>
+        <v>0.47484792715285629</v>
       </c>
       <c r="H17">
-        <v>0.4752021309977378</v>
-      </c>
-    </row>
-    <row r="18" spans="1:8">
+        <v>0.47520213099773778</v>
+      </c>
+    </row>
+    <row r="18" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A18">
         <v>2016</v>
       </c>
@@ -2058,16 +2083,16 @@
         <v>90272.72</v>
       </c>
       <c r="F18">
-        <v>365.4765991902834</v>
+        <v>365.47659919028342</v>
       </c>
       <c r="G18">
-        <v>0.0002489569652567896</v>
+        <v>2.4895696525678958E-4</v>
       </c>
       <c r="H18">
-        <v>0.0009009217688117088</v>
-      </c>
-    </row>
-    <row r="19" spans="1:8">
+        <v>9.009217688117088E-4</v>
+      </c>
+    </row>
+    <row r="19" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A19">
         <v>2016</v>
       </c>
@@ -2084,16 +2109,16 @@
         <v>1564686.97</v>
       </c>
       <c r="F19">
-        <v>142.1318566224895</v>
+        <v>142.13185662248949</v>
       </c>
       <c r="G19">
-        <v>0.009955113903086116</v>
+        <v>9.9551139030861161E-3</v>
       </c>
       <c r="H19">
-        <v>0.01561557636292596</v>
-      </c>
-    </row>
-    <row r="20" spans="1:8">
+        <v>1.5615576362925959E-2</v>
+      </c>
+    </row>
+    <row r="20" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A20">
         <v>2016</v>
       </c>
@@ -2110,16 +2135,16 @@
         <v>14126885.25</v>
       </c>
       <c r="F20">
-        <v>260.6162313188465</v>
+        <v>260.61623131884647</v>
       </c>
       <c r="G20">
-        <v>0.05056569140940235</v>
+        <v>5.0565691409402348E-2</v>
       </c>
       <c r="H20">
         <v>0.1409863184274279</v>
       </c>
     </row>
-    <row r="21" spans="1:8">
+    <row r="21" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A21">
         <v>2016</v>
       </c>
@@ -2133,19 +2158,19 @@
         <v>869.1</v>
       </c>
       <c r="E21">
-        <v>844999.8100000001</v>
+        <v>844999.81</v>
       </c>
       <c r="F21">
         <v>972.2699459210678</v>
       </c>
       <c r="G21">
-        <v>0.0007806277724153573</v>
+        <v>7.8062777241535725E-4</v>
       </c>
       <c r="H21">
-        <v>0.00843309832107372</v>
-      </c>
-    </row>
-    <row r="22" spans="1:8">
+        <v>8.4330983210737197E-3</v>
+      </c>
+    </row>
+    <row r="22" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A22">
         <v>2016</v>
       </c>
@@ -2159,19 +2184,19 @@
         <v>465231.3</v>
       </c>
       <c r="E22">
-        <v>37090409.16</v>
+        <v>37090409.159999996</v>
       </c>
       <c r="F22">
         <v>79.72466418317083</v>
       </c>
       <c r="G22">
-        <v>0.437780274380113</v>
+        <v>0.43778027438011302</v>
       </c>
       <c r="H22">
-        <v>0.3701622929538094</v>
-      </c>
-    </row>
-    <row r="23" spans="1:8">
+        <v>0.37016229295380942</v>
+      </c>
+    </row>
+    <row r="23" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A23">
         <v>2016</v>
       </c>
@@ -2185,19 +2210,19 @@
         <v>525615.9</v>
       </c>
       <c r="E23">
-        <v>46483144.31</v>
+        <v>46483144.310000002</v>
       </c>
       <c r="F23">
         <v>88.43557493218907</v>
       </c>
       <c r="G23">
-        <v>0.5006693355697264</v>
+        <v>0.50066933556972637</v>
       </c>
       <c r="H23">
-        <v>0.4639017921659513</v>
-      </c>
-    </row>
-    <row r="24" spans="1:8">
+        <v>0.46390179216595129</v>
+      </c>
+    </row>
+    <row r="24" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A24">
         <v>2017</v>
       </c>
@@ -2214,16 +2239,16 @@
         <v>149428.99</v>
       </c>
       <c r="F24">
-        <v>361.3760338573156</v>
+        <v>361.37603385731558</v>
       </c>
       <c r="G24">
-        <v>0.0003578054846068904</v>
+        <v>3.5780548460689042E-4</v>
       </c>
       <c r="H24">
-        <v>0.001396596855970543</v>
-      </c>
-    </row>
-    <row r="25" spans="1:8">
+        <v>1.3965968559705431E-3</v>
+      </c>
+    </row>
+    <row r="25" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A25">
         <v>2017</v>
       </c>
@@ -2243,13 +2268,13 @@
         <v>133.4384374906958</v>
       </c>
       <c r="G25">
-        <v>0.01104245647011343</v>
+        <v>1.104245647011343E-2</v>
       </c>
       <c r="H25">
-        <v>0.01675515124603022</v>
-      </c>
-    </row>
-    <row r="26" spans="1:8">
+        <v>1.675515124603022E-2</v>
+      </c>
+    </row>
+    <row r="26" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A26">
         <v>2017</v>
       </c>
@@ -2263,19 +2288,19 @@
         <v>65711.5</v>
       </c>
       <c r="E26">
-        <v>18559321.3</v>
+        <v>18559321.300000001</v>
       </c>
       <c r="F26">
-        <v>282.4364274137708</v>
+        <v>282.43642741377079</v>
       </c>
       <c r="G26">
-        <v>0.05491333259841519</v>
+        <v>5.4913332598415188E-2</v>
       </c>
       <c r="H26">
         <v>0.1734595795402695</v>
       </c>
     </row>
-    <row r="27" spans="1:8">
+    <row r="27" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A27">
         <v>2017</v>
       </c>
@@ -2295,13 +2320,13 @@
         <v>1069.49974313694</v>
       </c>
       <c r="G27">
-        <v>0.0005035434887809764</v>
+        <v>5.0354348878097637E-4</v>
       </c>
       <c r="H27">
-        <v>0.006226374151017454</v>
-      </c>
-    </row>
-    <row r="28" spans="1:8">
+        <v>6.2263741510174544E-3</v>
+      </c>
+    </row>
+    <row r="28" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A28">
         <v>2017</v>
       </c>
@@ -2315,19 +2340,19 @@
         <v>475875.5</v>
       </c>
       <c r="E28">
-        <v>37619223.37</v>
+        <v>37619223.369999997</v>
       </c>
       <c r="F28">
         <v>79.052658457937</v>
       </c>
       <c r="G28">
-        <v>0.4036559686252235</v>
+        <v>0.40365596862522352</v>
       </c>
       <c r="H28">
-        <v>0.3515976992322278</v>
-      </c>
-    </row>
-    <row r="29" spans="1:8">
+        <v>0.35159769923222778</v>
+      </c>
+    </row>
+    <row r="29" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A29">
         <v>2017</v>
       </c>
@@ -2341,19 +2366,19 @@
         <v>616003.5</v>
       </c>
       <c r="E29">
-        <v>48208194.56</v>
+        <v>48208194.560000002</v>
       </c>
       <c r="F29">
-        <v>78.25961144701289</v>
+        <v>78.259611447012887</v>
       </c>
       <c r="G29">
-        <v>0.52952689333286</v>
+        <v>0.52952689333285996</v>
       </c>
       <c r="H29">
-        <v>0.4505645989744844</v>
-      </c>
-    </row>
-    <row r="30" spans="1:8">
+        <v>0.45056459897448442</v>
+      </c>
+    </row>
+    <row r="30" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A30">
         <v>2018</v>
       </c>
@@ -2364,22 +2389,22 @@
         <v>596</v>
       </c>
       <c r="D30">
-        <v>649.2</v>
+        <v>649.20000000000005</v>
       </c>
       <c r="E30">
         <v>248162.95</v>
       </c>
       <c r="F30">
-        <v>382.2596272335182</v>
+        <v>382.25962723351819</v>
       </c>
       <c r="G30">
-        <v>0.0005048019710992401</v>
+        <v>5.0480197109924012E-4</v>
       </c>
       <c r="H30">
-        <v>0.002167330964225609</v>
-      </c>
-    </row>
-    <row r="31" spans="1:8">
+        <v>2.1673309642256089E-3</v>
+      </c>
+    </row>
+    <row r="31" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A31">
         <v>2018</v>
       </c>
@@ -2399,13 +2424,13 @@
         <v>120.8925120953663</v>
       </c>
       <c r="G31">
-        <v>0.0119229821261141</v>
+        <v>1.19229821261141E-2</v>
       </c>
       <c r="H31">
-        <v>0.01693442276150146</v>
-      </c>
-    </row>
-    <row r="32" spans="1:8">
+        <v>1.693442276150146E-2</v>
+      </c>
+    </row>
+    <row r="32" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A32">
         <v>2018</v>
       </c>
@@ -2422,16 +2447,16 @@
         <v>23598335.25</v>
       </c>
       <c r="F32">
-        <v>316.2849345270805</v>
+        <v>316.28493452708051</v>
       </c>
       <c r="G32">
-        <v>0.05662506002993239</v>
+        <v>5.6625060029932388E-2</v>
       </c>
       <c r="H32">
-        <v>0.2060960457292342</v>
-      </c>
-    </row>
-    <row r="33" spans="1:8">
+        <v>0.20609604572923421</v>
+      </c>
+    </row>
+    <row r="33" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A33">
         <v>2018</v>
       </c>
@@ -2445,19 +2470,19 @@
         <v>654</v>
       </c>
       <c r="E33">
-        <v>815422.1699999999</v>
+        <v>815422.16999999993</v>
       </c>
       <c r="F33">
-        <v>1246.822889908257</v>
+        <v>1246.8228899082569</v>
       </c>
       <c r="G33">
-        <v>0.0005090368869641666</v>
+        <v>5.0903688696416665E-4</v>
       </c>
       <c r="H33">
-        <v>0.007121488997277949</v>
-      </c>
-    </row>
-    <row r="34" spans="1:8">
+        <v>7.1214889972779491E-3</v>
+      </c>
+    </row>
+    <row r="34" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A34">
         <v>2018</v>
       </c>
@@ -2471,19 +2496,19 @@
         <v>489072.1</v>
       </c>
       <c r="E34">
-        <v>36580128.48</v>
+        <v>36580128.479999997</v>
       </c>
       <c r="F34">
-        <v>74.79496066121949</v>
+        <v>74.794960661219491</v>
       </c>
       <c r="G34">
-        <v>0.3753355112093988</v>
+        <v>0.37533551120939879</v>
       </c>
       <c r="H34">
-        <v>0.3194725285545447</v>
-      </c>
-    </row>
-    <row r="35" spans="1:8">
+        <v>0.31947252855454472</v>
+      </c>
+    </row>
+    <row r="35" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A35">
         <v>2018</v>
       </c>
@@ -2497,19 +2522,19 @@
         <v>711949</v>
       </c>
       <c r="E35">
-        <v>51320572.05</v>
+        <v>51320572.049999997</v>
       </c>
       <c r="F35">
-        <v>72.08461849093123</v>
+        <v>72.084618490931234</v>
       </c>
       <c r="G35">
-        <v>0.5551026077764913</v>
+        <v>0.55510260777649134</v>
       </c>
       <c r="H35">
-        <v>0.448208182993216</v>
-      </c>
-    </row>
-    <row r="36" spans="1:8">
+        <v>0.44820818299321602</v>
+      </c>
+    </row>
+    <row r="36" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A36">
         <v>2019</v>
       </c>
@@ -2526,16 +2551,16 @@
         <v>321457.67</v>
       </c>
       <c r="F36">
-        <v>399.7732495958214</v>
+        <v>399.77324959582143</v>
       </c>
       <c r="G36">
-        <v>0.0005862681919019948</v>
+        <v>5.8626819190199476E-4</v>
       </c>
       <c r="H36">
-        <v>0.00265163191570276</v>
-      </c>
-    </row>
-    <row r="37" spans="1:8">
+        <v>2.6516319157027599E-3</v>
+      </c>
+    </row>
+    <row r="37" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A37">
         <v>2019</v>
       </c>
@@ -2555,13 +2580,13 @@
         <v>116.1605571743689</v>
       </c>
       <c r="G37">
-        <v>0.01269153381829438</v>
+        <v>1.269153381829438E-2</v>
       </c>
       <c r="H37">
-        <v>0.01759270561402016</v>
-      </c>
-    </row>
-    <row r="38" spans="1:8">
+        <v>1.7592705614020161E-2</v>
+      </c>
+    </row>
+    <row r="38" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A38">
         <v>2019</v>
       </c>
@@ -2575,19 +2600,19 @@
         <v>85573.7</v>
       </c>
       <c r="E38">
-        <v>27530023.47</v>
+        <v>27530023.469999999</v>
       </c>
       <c r="F38">
-        <v>321.7112672468293</v>
+        <v>321.71126724682932</v>
       </c>
       <c r="G38">
-        <v>0.05992286273976415</v>
+        <v>5.9922862739764153E-2</v>
       </c>
       <c r="H38">
-        <v>0.2270889628270436</v>
-      </c>
-    </row>
-    <row r="39" spans="1:8">
+        <v>0.22708896282704361</v>
+      </c>
+    </row>
+    <row r="39" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A39">
         <v>2019</v>
       </c>
@@ -2601,19 +2626,19 @@
         <v>600.4</v>
       </c>
       <c r="E39">
-        <v>803072.8200000001</v>
+        <v>803072.82000000007</v>
       </c>
       <c r="F39">
-        <v>1337.562991339107</v>
+        <v>1337.5629913391069</v>
       </c>
       <c r="G39">
-        <v>0.000438528607542692</v>
+        <v>4.3852860754269198E-4</v>
       </c>
       <c r="H39">
-        <v>0.006624366810552127</v>
-      </c>
-    </row>
-    <row r="40" spans="1:8">
+        <v>6.6243668105521267E-3</v>
+      </c>
+    </row>
+    <row r="40" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A40">
         <v>2019</v>
       </c>
@@ -2627,7 +2652,7 @@
         <v>504034</v>
       </c>
       <c r="E40">
-        <v>35536274.21</v>
+        <v>35536274.210000001</v>
       </c>
       <c r="F40">
         <v>70.50372437176857</v>
@@ -2636,10 +2661,10 @@
         <v>0.3575243223130547</v>
       </c>
       <c r="H40">
-        <v>0.293130721878252</v>
-      </c>
-    </row>
-    <row r="41" spans="1:8">
+        <v>0.29313072187825201</v>
+      </c>
+    </row>
+    <row r="41" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A41">
         <v>2019</v>
       </c>
@@ -2653,19 +2678,19 @@
         <v>788823</v>
       </c>
       <c r="E41">
-        <v>54906531.45</v>
+        <v>54906531.450000003</v>
       </c>
       <c r="F41">
-        <v>69.60564214025199</v>
+        <v>69.605642140251987</v>
       </c>
       <c r="G41">
-        <v>0.5688364843294421</v>
+        <v>0.56883648432944212</v>
       </c>
       <c r="H41">
-        <v>0.4529116109544294</v>
-      </c>
-    </row>
-    <row r="42" spans="1:8">
+        <v>0.45291161095442939</v>
+      </c>
+    </row>
+    <row r="42" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A42">
         <v>2020</v>
       </c>
@@ -2682,16 +2707,16 @@
         <v>339332.07</v>
       </c>
       <c r="F42">
-        <v>388.2962238242362</v>
+        <v>388.29622382423622</v>
       </c>
       <c r="G42">
-        <v>0.0005738401944609019</v>
+        <v>5.7384019446090186E-4</v>
       </c>
       <c r="H42">
-        <v>0.002783029250502715</v>
-      </c>
-    </row>
-    <row r="43" spans="1:8">
+        <v>2.7830292505027152E-3</v>
+      </c>
+    </row>
+    <row r="43" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A43">
         <v>2020</v>
       </c>
@@ -2708,16 +2733,16 @@
         <v>2081527.19</v>
       </c>
       <c r="F43">
-        <v>99.64609415391686</v>
+        <v>99.646094153916863</v>
       </c>
       <c r="G43">
-        <v>0.01311450511835364</v>
+        <v>1.311450511835364E-2</v>
       </c>
       <c r="H43">
-        <v>0.01707162855396109</v>
-      </c>
-    </row>
-    <row r="44" spans="1:8">
+        <v>1.7071628553961091E-2</v>
+      </c>
+    </row>
+    <row r="44" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A44">
         <v>2020</v>
       </c>
@@ -2731,19 +2756,19 @@
         <v>97966.7</v>
       </c>
       <c r="E44">
-        <v>33079075.19</v>
+        <v>33079075.190000001</v>
       </c>
       <c r="F44">
         <v>337.6563178100314</v>
       </c>
       <c r="G44">
-        <v>0.06207073923655613</v>
+        <v>6.2070739236556129E-2</v>
       </c>
       <c r="H44">
-        <v>0.2712977698610941</v>
-      </c>
-    </row>
-    <row r="45" spans="1:8">
+        <v>0.27129776986109411</v>
+      </c>
+    </row>
+    <row r="45" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A45">
         <v>2020</v>
       </c>
@@ -2760,16 +2785,16 @@
         <v>779925.6100000001</v>
       </c>
       <c r="F45">
-        <v>1239.94532591415</v>
+        <v>1239.9453259141501</v>
       </c>
       <c r="G45">
-        <v>0.0004362904849272025</v>
+        <v>4.3629048492720249E-4</v>
       </c>
       <c r="H45">
-        <v>0.006396553635045969</v>
-      </c>
-    </row>
-    <row r="46" spans="1:8">
+        <v>6.3965536350459691E-3</v>
+      </c>
+    </row>
+    <row r="46" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A46">
         <v>2020</v>
       </c>
@@ -2786,16 +2811,16 @@
         <v>30788682.16</v>
       </c>
       <c r="F46">
-        <v>59.62646970820512</v>
+        <v>59.626469708205121</v>
       </c>
       <c r="G46">
-        <v>0.3338610848230373</v>
+        <v>0.33386108482303728</v>
       </c>
       <c r="H46">
-        <v>0.2525131297955749</v>
-      </c>
-    </row>
-    <row r="47" spans="1:8">
+        <v>0.25251312979557489</v>
+      </c>
+    </row>
+    <row r="47" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A47">
         <v>2020</v>
       </c>
@@ -2809,19 +2834,19 @@
         <v>898338.1</v>
       </c>
       <c r="E47">
-        <v>54860492.46</v>
+        <v>54860492.460000001</v>
       </c>
       <c r="F47">
-        <v>61.06886979412317</v>
+        <v>61.068869794123167</v>
       </c>
       <c r="G47">
-        <v>0.5899435401426648</v>
+        <v>0.58994354014266481</v>
       </c>
       <c r="H47">
-        <v>0.4499378889038211</v>
-      </c>
-    </row>
-    <row r="48" spans="1:8">
+        <v>0.44993788890382108</v>
+      </c>
+    </row>
+    <row r="48" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A48">
         <v>2021</v>
       </c>
@@ -2835,19 +2860,19 @@
         <v>814</v>
       </c>
       <c r="E48">
-        <v>310375.6</v>
+        <v>310375.59999999998</v>
       </c>
       <c r="F48">
-        <v>381.2968058968059</v>
+        <v>381.29680589680589</v>
       </c>
       <c r="G48">
-        <v>0.0005162052301068347</v>
+        <v>5.1620523010683468E-4</v>
       </c>
       <c r="H48">
-        <v>0.002473838513270051</v>
-      </c>
-    </row>
-    <row r="49" spans="1:8">
+        <v>2.4738385132700509E-3</v>
+      </c>
+    </row>
+    <row r="49" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A49">
         <v>2021</v>
       </c>
@@ -2864,16 +2889,16 @@
         <v>2055491.52</v>
       </c>
       <c r="F49">
-        <v>88.02773045545064</v>
+        <v>88.027730455450637</v>
       </c>
       <c r="G49">
-        <v>0.0139573165783708</v>
+        <v>1.39573165783708E-2</v>
       </c>
       <c r="H49">
-        <v>0.01638322756645818</v>
-      </c>
-    </row>
-    <row r="50" spans="1:8">
+        <v>1.6383227566458179E-2</v>
+      </c>
+    </row>
+    <row r="50" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A50">
         <v>2021</v>
       </c>
@@ -2887,19 +2912,19 @@
         <v>108975</v>
       </c>
       <c r="E50">
-        <v>38881379.67</v>
+        <v>38881379.670000002</v>
       </c>
       <c r="F50">
-        <v>356.7917381968342</v>
+        <v>356.79173819683422</v>
       </c>
       <c r="G50">
-        <v>0.06578241233546385</v>
+        <v>6.578241233546385E-2</v>
       </c>
       <c r="H50">
-        <v>0.3099027580670684</v>
-      </c>
-    </row>
-    <row r="51" spans="1:8">
+        <v>0.30990275806706841</v>
+      </c>
+    </row>
+    <row r="51" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A51">
         <v>2021</v>
       </c>
@@ -2913,19 +2938,19 @@
         <v>635.9</v>
       </c>
       <c r="E51">
-        <v>868273.0299999999</v>
+        <v>868273.02999999991</v>
       </c>
       <c r="F51">
-        <v>1365.423855952194</v>
+        <v>1365.4238559521939</v>
       </c>
       <c r="G51">
-        <v>0.0004173284026755388</v>
+        <v>4.1732840267553881E-4</v>
       </c>
       <c r="H51">
-        <v>0.006920541632936616</v>
-      </c>
-    </row>
-    <row r="52" spans="1:8">
+        <v>6.920541632936616E-3</v>
+      </c>
+    </row>
+    <row r="52" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A52">
         <v>2021</v>
       </c>
@@ -2939,19 +2964,19 @@
         <v>513143.8</v>
       </c>
       <c r="E52">
-        <v>28587944.03</v>
+        <v>28587944.030000001</v>
       </c>
       <c r="F52">
         <v>55.71136985383044</v>
       </c>
       <c r="G52">
-        <v>0.3125291942356855</v>
+        <v>0.31252919423568548</v>
       </c>
       <c r="H52">
-        <v>0.2278592677923864</v>
-      </c>
-    </row>
-    <row r="53" spans="1:8">
+        <v>0.22785926779238641</v>
+      </c>
+    </row>
+    <row r="53" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A53">
         <v>2021</v>
       </c>
@@ -2962,22 +2987,22 @@
         <v>889851</v>
       </c>
       <c r="D53">
-        <v>974801.7000000001</v>
+        <v>974801.70000000007</v>
       </c>
       <c r="E53">
-        <v>54759697.28</v>
+        <v>54759697.280000001</v>
       </c>
       <c r="F53">
         <v>56.17521725700724</v>
       </c>
       <c r="G53">
-        <v>0.6067975432176974</v>
+        <v>0.60679754321769741</v>
       </c>
       <c r="H53">
-        <v>0.4364603664278804</v>
-      </c>
-    </row>
-    <row r="54" spans="1:8">
+        <v>0.43646036642788039</v>
+      </c>
+    </row>
+    <row r="54" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A54">
         <v>2022</v>
       </c>
@@ -2994,16 +3019,16 @@
         <v>327104.08</v>
       </c>
       <c r="F54">
-        <v>355.084759009987</v>
+        <v>355.08475900998701</v>
       </c>
       <c r="G54">
-        <v>0.0005315952626977188</v>
+        <v>5.3159526269771877E-4</v>
       </c>
       <c r="H54">
-        <v>0.002441707993600441</v>
-      </c>
-    </row>
-    <row r="55" spans="1:8">
+        <v>2.4417079936004411E-3</v>
+      </c>
+    </row>
+    <row r="55" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A55">
         <v>2022</v>
       </c>
@@ -3020,16 +3045,16 @@
         <v>2138353.04</v>
       </c>
       <c r="F55">
-        <v>77.22557629732356</v>
+        <v>77.225576297323556</v>
       </c>
       <c r="G55">
-        <v>0.01550719338685319</v>
+        <v>1.5507193386853191E-2</v>
       </c>
       <c r="H55">
-        <v>0.01596199506563111</v>
-      </c>
-    </row>
-    <row r="56" spans="1:8">
+        <v>1.5961995065631111E-2</v>
+      </c>
+    </row>
+    <row r="56" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A56">
         <v>2022</v>
       </c>
@@ -3043,19 +3068,19 @@
         <v>125866.6</v>
       </c>
       <c r="E56">
-        <v>47273395.34</v>
+        <v>47273395.340000004</v>
       </c>
       <c r="F56">
-        <v>375.5833186881985</v>
+        <v>375.58331868819852</v>
       </c>
       <c r="G56">
-        <v>0.0706379461092123</v>
+        <v>7.0637946109212299E-2</v>
       </c>
       <c r="H56">
-        <v>0.3528779808748085</v>
-      </c>
-    </row>
-    <row r="57" spans="1:8">
+        <v>0.35287798087480848</v>
+      </c>
+    </row>
+    <row r="57" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A57">
         <v>2022</v>
       </c>
@@ -3069,19 +3094,19 @@
         <v>491.8</v>
       </c>
       <c r="E57">
-        <v>1069174.14</v>
+        <v>1069174.1399999999</v>
       </c>
       <c r="F57">
-        <v>2174.001911346076</v>
+        <v>2174.0019113460762</v>
       </c>
       <c r="G57">
-        <v>0.0003045862808997695</v>
+        <v>3.0458628089976951E-4</v>
       </c>
       <c r="H57">
-        <v>0.007980979767017509</v>
-      </c>
-    </row>
-    <row r="58" spans="1:8">
+        <v>7.9809797670175094E-3</v>
+      </c>
+    </row>
+    <row r="58" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A58">
         <v>2022</v>
       </c>
@@ -3095,19 +3120,19 @@
         <v>526179.5</v>
       </c>
       <c r="E58">
-        <v>28669623.39</v>
+        <v>28669623.390000001</v>
       </c>
       <c r="F58">
-        <v>54.48639369264671</v>
+        <v>54.486393692646708</v>
       </c>
       <c r="G58">
-        <v>0.2976780860027025</v>
+        <v>0.29767808600270251</v>
       </c>
       <c r="H58">
         <v>0.2140078735944754</v>
       </c>
     </row>
-    <row r="59" spans="1:8">
+    <row r="59" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A59">
         <v>2022</v>
       </c>
@@ -3118,22 +3143,22 @@
         <v>967700</v>
       </c>
       <c r="D59">
-        <v>1057888.4</v>
+        <v>1057888.3999999999</v>
       </c>
       <c r="E59">
-        <v>54487623.85</v>
+        <v>54487623.850000001</v>
       </c>
       <c r="F59">
-        <v>51.5060226107026</v>
+        <v>51.506022610702601</v>
       </c>
       <c r="G59">
-        <v>0.6153405929576345</v>
+        <v>0.61534059295763455</v>
       </c>
       <c r="H59">
-        <v>0.4067294627044671</v>
-      </c>
-    </row>
-    <row r="60" spans="1:8">
+        <v>0.40672946270446708</v>
+      </c>
+    </row>
+    <row r="60" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A60">
         <v>2023</v>
       </c>
@@ -3150,16 +3175,16 @@
         <v>684010.5</v>
       </c>
       <c r="F60">
-        <v>416.1407191093265</v>
+        <v>416.14071910932648</v>
       </c>
       <c r="G60">
-        <v>0.0009028544135347167</v>
+        <v>9.028544135347167E-4</v>
       </c>
       <c r="H60">
-        <v>0.004436445140940131</v>
-      </c>
-    </row>
-    <row r="61" spans="1:8">
+        <v>4.4364451409401309E-3</v>
+      </c>
+    </row>
+    <row r="61" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A61">
         <v>2023</v>
       </c>
@@ -3170,22 +3195,22 @@
         <v>31941</v>
       </c>
       <c r="D61">
-        <v>35419.8</v>
+        <v>35419.800000000003</v>
       </c>
       <c r="E61">
         <v>2629298.46</v>
       </c>
       <c r="F61">
-        <v>74.23244795283993</v>
+        <v>74.232447952839934</v>
       </c>
       <c r="G61">
-        <v>0.01902247547672321</v>
+        <v>1.902247547672321E-2</v>
       </c>
       <c r="H61">
-        <v>0.0170534492920041</v>
-      </c>
-    </row>
-    <row r="62" spans="1:8">
+        <v>1.70534492920041E-2</v>
+      </c>
+    </row>
+    <row r="62" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A62">
         <v>2023</v>
       </c>
@@ -3199,19 +3224,19 @@
         <v>163714.9</v>
       </c>
       <c r="E62">
-        <v>59012116.73999999</v>
+        <v>59012116.739999987</v>
       </c>
       <c r="F62">
-        <v>360.456603155852</v>
+        <v>360.45660315585201</v>
       </c>
       <c r="G62">
-        <v>0.08779782731301355</v>
+        <v>8.7797827313013554E-2</v>
       </c>
       <c r="H62">
         <v>0.3827485375849709</v>
       </c>
     </row>
-    <row r="63" spans="1:8">
+    <row r="63" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A63">
         <v>2023</v>
       </c>
@@ -3228,16 +3253,16 @@
         <v>22969.48</v>
       </c>
       <c r="F63">
-        <v>876.6977099236641</v>
+        <v>876.69770992366409</v>
       </c>
       <c r="G63">
-        <v>1.488876011765694E-05</v>
+        <v>1.488876011765694E-5</v>
       </c>
       <c r="H63">
-        <v>0.0001489784702660581</v>
-      </c>
-    </row>
-    <row r="64" spans="1:8">
+        <v>1.4897847026605811E-4</v>
+      </c>
+    </row>
+    <row r="64" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A64">
         <v>2023</v>
       </c>
@@ -3251,19 +3276,19 @@
         <v>551471.4</v>
       </c>
       <c r="E64">
-        <v>30285895.8</v>
+        <v>30285895.800000001</v>
       </c>
       <c r="F64">
-        <v>54.9183435441983</v>
+        <v>54.918343544198301</v>
       </c>
       <c r="G64">
-        <v>0.2965614706283474</v>
+        <v>0.29656147062834742</v>
       </c>
       <c r="H64">
-        <v>0.1964322408222229</v>
-      </c>
-    </row>
-    <row r="65" spans="1:8">
+        <v>0.19643224082222291</v>
+      </c>
+    </row>
+    <row r="65" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A65">
         <v>2023</v>
       </c>
@@ -3277,19 +3302,19 @@
         <v>1075270.2</v>
       </c>
       <c r="E65">
-        <v>61545571.11</v>
+        <v>61545571.109999999</v>
       </c>
       <c r="F65">
         <v>57.23730752512251</v>
       </c>
       <c r="G65">
-        <v>0.5957004834082635</v>
+        <v>0.59570048340826354</v>
       </c>
       <c r="H65">
-        <v>0.3991803486895958</v>
-      </c>
-    </row>
-    <row r="66" spans="1:8">
+        <v>0.39918034868959579</v>
+      </c>
+    </row>
+    <row r="66" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A66">
         <v>2024</v>
       </c>
@@ -3306,16 +3331,16 @@
         <v>690636.96</v>
       </c>
       <c r="F66">
-        <v>360.213299953059</v>
+        <v>360.21329995305899</v>
       </c>
       <c r="G66">
-        <v>0.0008909774493152223</v>
+        <v>8.9097744931522233E-4</v>
       </c>
       <c r="H66">
-        <v>0.005023226958853812</v>
-      </c>
-    </row>
-    <row r="67" spans="1:8">
+        <v>5.0232269588538119E-3</v>
+      </c>
+    </row>
+    <row r="67" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A67">
         <v>2024</v>
       </c>
@@ -3332,16 +3357,16 @@
         <v>2035881.97</v>
       </c>
       <c r="F67">
-        <v>60.37269459905877</v>
+        <v>60.372694599058768</v>
       </c>
       <c r="G67">
-        <v>0.01531762764225915</v>
+        <v>1.5317627642259151E-2</v>
       </c>
       <c r="H67">
-        <v>0.01480763091038222</v>
-      </c>
-    </row>
-    <row r="68" spans="1:8">
+        <v>1.480763091038222E-2</v>
+      </c>
+    </row>
+    <row r="68" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A68">
         <v>2024</v>
       </c>
@@ -3355,19 +3380,19 @@
         <v>178210.3</v>
       </c>
       <c r="E68">
-        <v>53347495.11</v>
+        <v>53347495.109999999</v>
       </c>
       <c r="F68">
-        <v>299.351356851989</v>
+        <v>299.35135685198901</v>
       </c>
       <c r="G68">
-        <v>0.08128638727111467</v>
+        <v>8.1286387271114674E-2</v>
       </c>
       <c r="H68">
         <v>0.3880136615102005</v>
       </c>
     </row>
-    <row r="69" spans="1:8">
+    <row r="69" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A69">
         <v>2024</v>
       </c>
@@ -3384,16 +3409,16 @@
         <v>26055.67</v>
       </c>
       <c r="F69">
-        <v>845.9633116883116</v>
+        <v>845.96331168831159</v>
       </c>
       <c r="G69">
-        <v>1.366064232340205E-05</v>
+        <v>1.3660642323402051E-5</v>
       </c>
       <c r="H69">
-        <v>0.0001895113519192464</v>
-      </c>
-    </row>
-    <row r="70" spans="1:8">
+        <v>1.8951135191924641E-4</v>
+      </c>
+    </row>
+    <row r="70" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A70">
         <v>2024</v>
       </c>
@@ -3404,22 +3429,22 @@
         <v>533212</v>
       </c>
       <c r="D70">
-        <v>590941.8</v>
+        <v>590941.80000000005</v>
       </c>
       <c r="E70">
-        <v>25623936.89</v>
+        <v>25623936.890000001</v>
       </c>
       <c r="F70">
-        <v>43.36118529777382</v>
+        <v>43.361185297773822</v>
       </c>
       <c r="G70">
-        <v>0.2697784597979945</v>
+        <v>0.26977845979799447</v>
       </c>
       <c r="H70">
-        <v>0.1863712167646178</v>
-      </c>
-    </row>
-    <row r="71" spans="1:8">
+        <v>0.18637121676461779</v>
+      </c>
+    </row>
+    <row r="71" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A71">
         <v>2024</v>
       </c>
@@ -3433,16 +3458,16 @@
         <v>1346065.4</v>
       </c>
       <c r="E71">
-        <v>55764696.51</v>
+        <v>55764696.509999998</v>
       </c>
       <c r="F71">
-        <v>41.42792505475587</v>
+        <v>41.427925054755868</v>
       </c>
       <c r="G71">
-        <v>0.632712887196993</v>
+        <v>0.63271288719699303</v>
       </c>
       <c r="H71">
-        <v>0.4055947525040262</v>
+        <v>0.40559475250402621</v>
       </c>
     </row>
   </sheetData>

</xml_diff>